<commit_message>
cambios en el manejo de sesiones2
</commit_message>
<xml_diff>
--- a/app/fixtures/ejemplo_movimientos.xlsx
+++ b/app/fixtures/ejemplo_movimientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Fecha</t>
   </si>
@@ -36,82 +36,25 @@
     <t xml:space="preserve">Método de Pago</t>
   </si>
   <si>
+    <t>Gasto</t>
+  </si>
+  <si>
+    <t>Mantenimiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reparación de equipo de oficina</t>
+  </si>
+  <si>
+    <t>Tarjeta</t>
+  </si>
+  <si>
     <t>Ingreso</t>
   </si>
   <si>
     <t>Ventas</t>
   </si>
   <si>
-    <t xml:space="preserve">Venta de productos al contado</t>
-  </si>
-  <si>
-    <t>Efectivo</t>
-  </si>
-  <si>
-    <t>Gasto</t>
-  </si>
-  <si>
-    <t>Alquiler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pago de renta de local comercial</t>
-  </si>
-  <si>
-    <t>Transferencia</t>
-  </si>
-  <si>
-    <t>Servicios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consultoría y soporte técnico</t>
-  </si>
-  <si>
-    <t>Tarjeta</t>
-  </si>
-  <si>
-    <t>Compras</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adquisición de inventario y suministros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Servicios básicos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pago de factura de energía eléctrica y agua</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cobro por factura #1042</t>
-  </si>
-  <si>
-    <t>Pasivo</t>
-  </si>
-  <si>
-    <t>Personal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pago de nómina quincenal</t>
-  </si>
-  <si>
-    <t>Publicidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campaña publicitaria en redes sociales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Otros ingresos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reembolso de proveedor</t>
-  </si>
-  <si>
-    <t>Mantenimiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reparación de equipo de oficina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pagara despues</t>
+    <t xml:space="preserve">vendi algo</t>
   </si>
 </sst>
 </file>
@@ -149,10 +92,16 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="3" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -681,7 +630,7 @@
     </row>
     <row r="4" ht="14.25">
       <c r="A4" s="2">
-        <v>46296</v>
+        <v>46317</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
@@ -692,8 +641,8 @@
       <c r="D4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="3">
-        <v>1250</v>
+      <c r="E4">
+        <v>100</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
@@ -701,183 +650,64 @@
     </row>
     <row r="5" ht="14.25">
       <c r="A5" s="2">
-        <v>46297</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5">
-        <v>-850</v>
+        <v>46317</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3">
+        <v>300</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" s="2">
-        <v>46298</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6">
-        <v>450.5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>16</v>
+        <v>46317</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="2">
-        <v>46300</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="3">
-        <v>1200</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
+      <c r="A7" s="2"/>
+      <c r="E7" s="5"/>
     </row>
     <row r="8" ht="14.25">
-      <c r="A8" s="2">
-        <v>46302</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8">
-        <v>-135.19999999999999</v>
-      </c>
-      <c r="F8" t="s">
-        <v>9</v>
-      </c>
+      <c r="A8" s="2"/>
     </row>
     <row r="9" ht="14.25">
-      <c r="A9" s="2">
-        <v>46305</v>
-      </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="3">
-        <v>2300</v>
-      </c>
-      <c r="F9" t="s">
-        <v>13</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" ht="14.25">
-      <c r="A10" s="2">
-        <v>46307</v>
-      </c>
-      <c r="B10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="3">
-        <v>3100</v>
-      </c>
-      <c r="F10" t="s">
-        <v>13</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" ht="14.25">
-      <c r="A11" s="2">
-        <v>46310</v>
-      </c>
-      <c r="B11" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11">
-        <v>250</v>
-      </c>
-      <c r="F11" t="s">
-        <v>16</v>
-      </c>
+      <c r="A11" s="2"/>
     </row>
     <row r="12" ht="14.25">
-      <c r="A12" s="2">
-        <v>46313</v>
-      </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12">
-        <v>85</v>
-      </c>
-      <c r="F12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" ht="14.25">
-      <c r="A13" s="2">
-        <v>46315</v>
-      </c>
-      <c r="B13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" t="s">
-        <v>30</v>
-      </c>
-      <c r="E13">
-        <v>175</v>
-      </c>
-      <c r="F13" t="s">
-        <v>31</v>
-      </c>
+      <c r="A12" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>